<commit_message>
Update eu-taxonomy-financial excel files
The tootltip for UN Global Compact Principles Compliance Policy is now the same as in sfdr.
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/euTaxonomyNonFinancials/EutaxonomyNonFinancials.xlsx
+++ b/dataland-framework-toolbox/inputs/euTaxonomyNonFinancials/EutaxonomyNonFinancials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\srv\data\dataland\dataland-framework-toolbox\inputs\euTaxonomyNonFinancials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F382588B-8A6C-4182-8104-9980D8AD69F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C74F531A-E514-478E-AD0B-63F5971F6317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
@@ -214,9 +214,6 @@
     <t>UNGC_PRINCIPLES_COMPLIANCE_POLICY</t>
   </si>
   <si>
-    <t>Does the company have a policy to monitor compliance with the UNGC principles or OECD Guidelines for Multinational Enterprises? (See Regulation (EU) 2022/1288, Annex I, top (22) and table 1, indicator nr. 11.) If yes, please share the relevant documents with us.</t>
-  </si>
-  <si>
     <t>OECD Guidelines for Multinational Enterprises Compliance Policy</t>
   </si>
   <si>
@@ -1132,6 +1129,10 @@
   <si>
     <t>Existence of policies in place to support/respect human rights and carry out due diligence to ensure that the business activities do not have a negative human rights impact.
 Linked to Regulation (EU) 2022/1288, Annex I, Table 3, Adverse impact on sustainability factor 10</t>
+  </si>
+  <si>
+    <t>Existence of a policy to monitor compliance with the UNGC principles or OECD Guidelines for Multinational Enterprises.
+Linked to Regulation (EU) 2022/1288, Annex I, Table 1, Adverse sustainability indicator 11</t>
   </si>
 </sst>
 </file>
@@ -1540,12 +1541,14 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1822,20 +1825,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q108"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="20.26953125" customWidth="1"/>
-    <col min="4" max="5" width="75.7265625" customWidth="1"/>
-    <col min="6" max="6" width="255.6328125" customWidth="1"/>
-    <col min="7" max="7" width="44.7265625" customWidth="1"/>
-    <col min="8" max="8" width="26.26953125" customWidth="1"/>
-    <col min="9" max="15" width="14.26953125" customWidth="1"/>
-    <col min="16" max="16" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.81640625" customWidth="1"/>
-    <col min="18" max="18" width="8.7265625" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
+    <col min="4" max="5" width="75.7109375" customWidth="1"/>
+    <col min="6" max="6" width="255.5703125" customWidth="1"/>
+    <col min="7" max="7" width="44.7109375" customWidth="1"/>
+    <col min="8" max="8" width="26.28515625" customWidth="1"/>
+    <col min="9" max="15" width="14.28515625" customWidth="1"/>
+    <col min="16" max="16" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.85546875" customWidth="1"/>
+    <col min="18" max="18" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1888,7 +1891,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="6">
         <v>0</v>
       </c>
@@ -1899,7 +1902,7 @@
       <c r="D2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="37" t="s">
+      <c r="E2" s="36" t="s">
         <v>19</v>
       </c>
       <c r="F2" s="23" t="s">
@@ -1922,7 +1925,7 @@
       <c r="O2" s="11"/>
       <c r="P2" s="11"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="7" t="s">
         <v>17</v>
@@ -1931,7 +1934,7 @@
       <c r="D3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="36" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="18" t="s">
@@ -1952,7 +1955,7 @@
       <c r="O3" s="11"/>
       <c r="P3" s="11"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
         <v>1</v>
       </c>
@@ -1963,7 +1966,7 @@
       <c r="D4" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="E4" s="36" t="s">
         <v>29</v>
       </c>
       <c r="F4" s="18" t="s">
@@ -1986,7 +1989,7 @@
       <c r="O4" s="11"/>
       <c r="P4" s="11"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
         <v>2</v>
       </c>
@@ -1997,7 +2000,7 @@
       <c r="D5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="E5" s="36" t="s">
         <v>34</v>
       </c>
       <c r="F5" s="11" t="s">
@@ -2025,7 +2028,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
         <v>3</v>
       </c>
@@ -2036,7 +2039,7 @@
       <c r="D6" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="36" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="18" t="s">
@@ -2059,7 +2062,7 @@
       <c r="O6" s="11"/>
       <c r="P6" s="11"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="6">
         <v>4</v>
       </c>
@@ -2070,7 +2073,7 @@
       <c r="D7" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="37" t="s">
+      <c r="E7" s="36" t="s">
         <v>43</v>
       </c>
       <c r="F7" s="18" t="s">
@@ -2091,7 +2094,7 @@
       <c r="O7" s="11"/>
       <c r="P7" s="11"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>5</v>
       </c>
@@ -2099,10 +2102,10 @@
         <v>17</v>
       </c>
       <c r="C8" s="7"/>
-      <c r="D8" s="35" t="s">
+      <c r="D8" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="37" t="s">
+      <c r="E8" s="36" t="s">
         <v>47</v>
       </c>
       <c r="F8" s="11" t="s">
@@ -2125,7 +2128,7 @@
       <c r="O8" s="11"/>
       <c r="P8" s="11"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" ht="24.75" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>6</v>
       </c>
@@ -2133,14 +2136,14 @@
         <v>17</v>
       </c>
       <c r="C9" s="7"/>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="33" t="s">
-        <v>53</v>
+      <c r="F9" s="37" t="s">
+        <v>358</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>36</v>
@@ -2157,7 +2160,7 @@
       <c r="O9" s="11"/>
       <c r="P9" s="11"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
         <v>7</v>
       </c>
@@ -2166,13 +2169,13 @@
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="E10" s="37" t="s">
+      <c r="F10" s="33" t="s">
         <v>55</v>
-      </c>
-      <c r="F10" s="34" t="s">
-        <v>56</v>
       </c>
       <c r="G10" s="19" t="s">
         <v>36</v>
@@ -2189,7 +2192,7 @@
       <c r="O10" s="11"/>
       <c r="P10" s="11"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="6">
         <v>8</v>
       </c>
@@ -2197,14 +2200,14 @@
         <v>17</v>
       </c>
       <c r="C11" s="7"/>
-      <c r="D11" s="36" t="s">
+      <c r="D11" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="37" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" s="34" t="s">
-        <v>357</v>
+      <c r="F11" s="33" t="s">
+        <v>356</v>
       </c>
       <c r="G11" s="19" t="s">
         <v>36</v>
@@ -2221,7 +2224,7 @@
       <c r="O11" s="11"/>
       <c r="P11" s="11"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>9</v>
       </c>
@@ -2229,14 +2232,14 @@
         <v>17</v>
       </c>
       <c r="C12" s="7"/>
-      <c r="D12" s="36" t="s">
+      <c r="D12" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="34" t="s">
-        <v>358</v>
+      <c r="F12" s="33" t="s">
+        <v>357</v>
       </c>
       <c r="G12" s="19" t="s">
         <v>36</v>
@@ -2253,7 +2256,7 @@
       <c r="O12" s="11"/>
       <c r="P12" s="11"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>10</v>
       </c>
@@ -2262,14 +2265,14 @@
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="36" t="s">
         <v>61</v>
-      </c>
-      <c r="E13" s="37" t="s">
-        <v>62</v>
       </c>
       <c r="F13" s="11"/>
       <c r="G13" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H13" s="22" t="s">
         <v>32</v>
@@ -2283,25 +2286,25 @@
       <c r="O13" s="11"/>
       <c r="P13" s="11"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>11</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="37" t="s">
+      <c r="F14" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="G14" s="20" t="s">
         <v>67</v>
-      </c>
-      <c r="G14" s="20" t="s">
-        <v>68</v>
       </c>
       <c r="H14" s="21"/>
       <c r="I14" s="11"/>
@@ -2315,27 +2318,27 @@
       <c r="O14" s="11"/>
       <c r="P14" s="11"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="E15" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="E15" s="37" t="s">
+      <c r="F15" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="F15" s="27" t="s">
-        <v>73</v>
-      </c>
       <c r="G15" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H15" s="21"/>
       <c r="I15" s="11"/>
@@ -2346,34 +2349,34 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
       <c r="N15" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="O15" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="P15" s="11"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="O15" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="P15" s="11"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A16" s="17" t="s">
+      <c r="B16" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D16" s="14" t="s">
+      <c r="E16" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="37" t="s">
+      <c r="F16" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="F16" s="27" t="s">
-        <v>79</v>
-      </c>
       <c r="G16" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H16" s="21"/>
       <c r="I16" s="11"/>
@@ -2384,34 +2387,34 @@
       <c r="L16" s="11"/>
       <c r="M16" s="11"/>
       <c r="N16" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P16" s="11"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="36" t="s">
         <v>81</v>
       </c>
-      <c r="D17" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E17" s="37" t="s">
+      <c r="F17" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="F17" s="11" t="s">
-        <v>83</v>
-      </c>
       <c r="G17" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H17" s="21"/>
       <c r="I17" s="11"/>
@@ -2422,34 +2425,34 @@
       <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P17" s="11"/>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="B18" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="37" t="s">
+      <c r="F18" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="11" t="s">
-        <v>86</v>
-      </c>
       <c r="G18" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H18" s="21"/>
       <c r="I18" s="11"/>
@@ -2460,34 +2463,34 @@
       <c r="L18" s="11"/>
       <c r="M18" s="11"/>
       <c r="N18" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O18" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P18" s="11"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E19" s="37" t="s">
+      <c r="F19" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="F19" s="27" t="s">
-        <v>90</v>
-      </c>
       <c r="G19" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H19" s="21"/>
       <c r="I19" s="11"/>
@@ -2498,34 +2501,34 @@
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
       <c r="N19" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O19" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P19" s="11"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E20" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="37" t="s">
+      <c r="F20" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="27" t="s">
-        <v>93</v>
-      </c>
       <c r="G20" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H20" s="21"/>
       <c r="I20" s="11"/>
@@ -2536,32 +2539,32 @@
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O20" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P20" s="11"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="E21" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="E21" s="37" t="s">
+      <c r="F21" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F21" s="27" t="s">
+      <c r="G21" s="20" t="s">
         <v>97</v>
-      </c>
-      <c r="G21" s="20" t="s">
-        <v>98</v>
       </c>
       <c r="H21" s="21"/>
       <c r="I21" s="11"/>
@@ -2572,34 +2575,34 @@
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
       <c r="N21" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P21" s="11"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C22" s="7" t="s">
+      <c r="D22" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E22" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="D22" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E22" s="37" t="s">
+      <c r="F22" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F22" s="11" t="s">
-        <v>102</v>
-      </c>
       <c r="G22" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H22" s="21"/>
       <c r="I22" s="11"/>
@@ -2610,34 +2613,34 @@
       <c r="L22" s="11"/>
       <c r="M22" s="11"/>
       <c r="N22" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O22" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P22" s="11"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E23" s="37" t="s">
+      <c r="F23" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="F23" s="11" t="s">
-        <v>105</v>
-      </c>
       <c r="G23" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H23" s="21"/>
       <c r="I23" s="11"/>
@@ -2648,32 +2651,32 @@
       <c r="L23" s="11"/>
       <c r="M23" s="11"/>
       <c r="N23" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O23" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P23" s="11"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>17</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="E24" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="E24" s="37" t="s">
+      <c r="F24" s="29" t="s">
         <v>107</v>
       </c>
-      <c r="F24" s="29" t="s">
-        <v>108</v>
-      </c>
       <c r="G24" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H24" s="21"/>
       <c r="I24" s="11"/>
@@ -2684,32 +2687,32 @@
       <c r="L24" s="11"/>
       <c r="M24" s="11"/>
       <c r="N24" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P24" s="11"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="E25" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="E25" s="37" t="s">
+      <c r="F25" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="F25" s="29" t="s">
-        <v>112</v>
-      </c>
       <c r="G25" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H25" s="21"/>
       <c r="I25" s="11"/>
@@ -2720,32 +2723,32 @@
       <c r="L25" s="11"/>
       <c r="M25" s="11"/>
       <c r="N25" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P25" s="11"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="E26" s="36" t="s">
         <v>114</v>
       </c>
-      <c r="E26" s="37" t="s">
+      <c r="F26" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="F26" s="29" t="s">
-        <v>116</v>
-      </c>
       <c r="G26" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H26" s="21"/>
       <c r="I26" s="11"/>
@@ -2756,32 +2759,32 @@
       <c r="L26" s="11"/>
       <c r="M26" s="11"/>
       <c r="N26" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P26" s="11"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="E27" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="E27" s="37" t="s">
+      <c r="F27" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="F27" s="29" t="s">
-        <v>120</v>
-      </c>
       <c r="G27" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H27" s="21"/>
       <c r="I27" s="11"/>
@@ -2792,32 +2795,32 @@
       <c r="L27" s="11"/>
       <c r="M27" s="11"/>
       <c r="N27" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P27" s="11"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="E28" s="37" t="s">
+      <c r="F28" s="29" t="s">
         <v>123</v>
       </c>
-      <c r="F28" s="29" t="s">
-        <v>124</v>
-      </c>
       <c r="G28" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H28" s="21"/>
       <c r="I28" s="11"/>
@@ -2828,32 +2831,32 @@
       <c r="L28" s="11"/>
       <c r="M28" s="11"/>
       <c r="N28" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P28" s="11"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>18</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="E29" s="36" t="s">
         <v>125</v>
       </c>
-      <c r="E29" s="37" t="s">
+      <c r="F29" s="29" t="s">
         <v>126</v>
       </c>
-      <c r="F29" s="29" t="s">
-        <v>127</v>
-      </c>
       <c r="G29" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H29" s="21"/>
       <c r="I29" s="11"/>
@@ -2864,32 +2867,32 @@
       <c r="L29" s="11"/>
       <c r="M29" s="11"/>
       <c r="N29" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P29" s="11"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="E30" s="36" t="s">
         <v>129</v>
       </c>
-      <c r="E30" s="37" t="s">
+      <c r="F30" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="F30" s="29" t="s">
-        <v>131</v>
-      </c>
       <c r="G30" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H30" s="21"/>
       <c r="I30" s="11"/>
@@ -2900,32 +2903,32 @@
       <c r="L30" s="11"/>
       <c r="M30" s="11"/>
       <c r="N30" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P30" s="11"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="E31" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E31" s="37" t="s">
+      <c r="F31" s="29" t="s">
         <v>134</v>
       </c>
-      <c r="F31" s="29" t="s">
-        <v>135</v>
-      </c>
       <c r="G31" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H31" s="21"/>
       <c r="I31" s="11"/>
@@ -2936,32 +2939,32 @@
       <c r="L31" s="11"/>
       <c r="M31" s="11"/>
       <c r="N31" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P31" s="11"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="E32" s="36" t="s">
         <v>137</v>
       </c>
-      <c r="E32" s="37" t="s">
+      <c r="F32" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="F32" s="29" t="s">
-        <v>139</v>
-      </c>
       <c r="G32" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H32" s="21"/>
       <c r="I32" s="11"/>
@@ -2972,32 +2975,32 @@
       <c r="L32" s="11"/>
       <c r="M32" s="11"/>
       <c r="N32" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P32" s="11"/>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="6">
         <v>19</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="30" t="s">
+        <v>139</v>
+      </c>
+      <c r="E33" s="36" t="s">
         <v>140</v>
       </c>
-      <c r="E33" s="37" t="s">
+      <c r="F33" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="F33" s="29" t="s">
-        <v>142</v>
-      </c>
       <c r="G33" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H33" s="21"/>
       <c r="I33" s="11"/>
@@ -3008,32 +3011,32 @@
       <c r="L33" s="11"/>
       <c r="M33" s="11"/>
       <c r="N33" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P33" s="11"/>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="E34" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="E34" s="37" t="s">
+      <c r="F34" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="F34" s="29" t="s">
-        <v>146</v>
-      </c>
       <c r="G34" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H34" s="21"/>
       <c r="I34" s="11"/>
@@ -3044,32 +3047,32 @@
       <c r="L34" s="11"/>
       <c r="M34" s="11"/>
       <c r="N34" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P34" s="11"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="E35" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="E35" s="37" t="s">
+      <c r="F35" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="F35" s="29" t="s">
-        <v>150</v>
-      </c>
       <c r="G35" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H35" s="21"/>
       <c r="I35" s="11"/>
@@ -3080,32 +3083,32 @@
       <c r="L35" s="11"/>
       <c r="M35" s="11"/>
       <c r="N35" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P35" s="11"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="17" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="E36" s="36" t="s">
         <v>152</v>
       </c>
-      <c r="E36" s="37" t="s">
+      <c r="F36" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="F36" s="29" t="s">
-        <v>154</v>
-      </c>
       <c r="G36" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H36" s="21"/>
       <c r="I36" s="11"/>
@@ -3116,32 +3119,32 @@
       <c r="L36" s="11"/>
       <c r="M36" s="11"/>
       <c r="N36" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P36" s="11"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>20</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="E37" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="E37" s="37" t="s">
+      <c r="F37" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="F37" s="29" t="s">
-        <v>157</v>
-      </c>
       <c r="G37" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H37" s="21"/>
       <c r="I37" s="11"/>
@@ -3152,32 +3155,32 @@
       <c r="L37" s="11"/>
       <c r="M37" s="11"/>
       <c r="N37" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P37" s="11"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C38" s="7"/>
       <c r="D38" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="E38" s="36" t="s">
         <v>159</v>
       </c>
-      <c r="E38" s="37" t="s">
+      <c r="F38" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="F38" s="29" t="s">
-        <v>161</v>
-      </c>
       <c r="G38" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H38" s="21"/>
       <c r="I38" s="11"/>
@@ -3188,32 +3191,32 @@
       <c r="L38" s="11"/>
       <c r="M38" s="11"/>
       <c r="N38" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O38" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P38" s="11"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C39" s="7"/>
       <c r="D39" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="E39" s="36" t="s">
         <v>163</v>
       </c>
-      <c r="E39" s="37" t="s">
+      <c r="F39" s="29" t="s">
         <v>164</v>
       </c>
-      <c r="F39" s="29" t="s">
-        <v>165</v>
-      </c>
       <c r="G39" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H39" s="21"/>
       <c r="I39" s="11"/>
@@ -3224,32 +3227,32 @@
       <c r="L39" s="11"/>
       <c r="M39" s="11"/>
       <c r="N39" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O39" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P39" s="11"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C40" s="7"/>
       <c r="D40" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="E40" s="36" t="s">
         <v>167</v>
       </c>
-      <c r="E40" s="37" t="s">
+      <c r="F40" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="F40" s="29" t="s">
-        <v>169</v>
-      </c>
       <c r="G40" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H40" s="21"/>
       <c r="I40" s="11"/>
@@ -3260,32 +3263,32 @@
       <c r="L40" s="11"/>
       <c r="M40" s="11"/>
       <c r="N40" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O40" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P40" s="11"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="6">
         <v>21</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C41" s="7"/>
       <c r="D41" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="E41" s="36" t="s">
         <v>170</v>
       </c>
-      <c r="E41" s="37" t="s">
+      <c r="F41" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="F41" s="29" t="s">
-        <v>172</v>
-      </c>
       <c r="G41" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H41" s="21"/>
       <c r="I41" s="11"/>
@@ -3296,32 +3299,32 @@
       <c r="L41" s="11"/>
       <c r="M41" s="11"/>
       <c r="N41" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O41" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P41" s="11"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C42" s="7"/>
       <c r="D42" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="E42" s="36" t="s">
         <v>174</v>
       </c>
-      <c r="E42" s="37" t="s">
+      <c r="F42" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="F42" s="29" t="s">
-        <v>176</v>
-      </c>
       <c r="G42" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H42" s="21"/>
       <c r="I42" s="11"/>
@@ -3332,32 +3335,32 @@
       <c r="L42" s="11"/>
       <c r="M42" s="11"/>
       <c r="N42" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O42" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P42" s="11"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C43" s="7"/>
       <c r="D43" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="E43" s="36" t="s">
         <v>178</v>
       </c>
-      <c r="E43" s="37" t="s">
+      <c r="F43" s="29" t="s">
         <v>179</v>
       </c>
-      <c r="F43" s="29" t="s">
-        <v>180</v>
-      </c>
       <c r="G43" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H43" s="21"/>
       <c r="I43" s="11"/>
@@ -3368,32 +3371,32 @@
       <c r="L43" s="11"/>
       <c r="M43" s="11"/>
       <c r="N43" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O43" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P43" s="11"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C44" s="7"/>
       <c r="D44" s="30" t="s">
+        <v>181</v>
+      </c>
+      <c r="E44" s="36" t="s">
         <v>182</v>
       </c>
-      <c r="E44" s="37" t="s">
+      <c r="F44" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="F44" s="29" t="s">
-        <v>184</v>
-      </c>
       <c r="G44" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H44" s="21"/>
       <c r="I44" s="11"/>
@@ -3404,32 +3407,32 @@
       <c r="L44" s="11"/>
       <c r="M44" s="11"/>
       <c r="N44" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O44" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P44" s="11"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
         <v>22</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C45" s="7"/>
       <c r="D45" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="E45" s="36" t="s">
         <v>185</v>
       </c>
-      <c r="E45" s="37" t="s">
+      <c r="F45" s="29" t="s">
         <v>186</v>
       </c>
-      <c r="F45" s="29" t="s">
-        <v>187</v>
-      </c>
       <c r="G45" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H45" s="21"/>
       <c r="I45" s="11"/>
@@ -3440,32 +3443,32 @@
       <c r="L45" s="11"/>
       <c r="M45" s="11"/>
       <c r="N45" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O45" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P45" s="11"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C46" s="7"/>
       <c r="D46" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="E46" s="36" t="s">
         <v>189</v>
       </c>
-      <c r="E46" s="37" t="s">
+      <c r="F46" s="29" t="s">
         <v>190</v>
       </c>
-      <c r="F46" s="29" t="s">
-        <v>191</v>
-      </c>
       <c r="G46" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H46" s="21"/>
       <c r="I46" s="11"/>
@@ -3476,32 +3479,32 @@
       <c r="L46" s="11"/>
       <c r="M46" s="11"/>
       <c r="N46" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O46" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P46" s="11"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="E47" s="36" t="s">
         <v>193</v>
       </c>
-      <c r="E47" s="37" t="s">
+      <c r="F47" s="29" t="s">
         <v>194</v>
       </c>
-      <c r="F47" s="29" t="s">
-        <v>195</v>
-      </c>
       <c r="G47" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H47" s="21"/>
       <c r="I47" s="11"/>
@@ -3512,32 +3515,32 @@
       <c r="L47" s="11"/>
       <c r="M47" s="11"/>
       <c r="N47" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O47" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P47" s="11"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="E48" s="36" t="s">
         <v>197</v>
       </c>
-      <c r="E48" s="37" t="s">
+      <c r="F48" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="F48" s="29" t="s">
-        <v>199</v>
-      </c>
       <c r="G48" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H48" s="21"/>
       <c r="I48" s="11"/>
@@ -3548,32 +3551,32 @@
       <c r="L48" s="11"/>
       <c r="M48" s="11"/>
       <c r="N48" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O48" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P48" s="11"/>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="6">
         <v>23</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C49" s="7"/>
       <c r="D49" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="E49" s="36" t="s">
         <v>200</v>
       </c>
-      <c r="E49" s="37" t="s">
+      <c r="F49" s="27" t="s">
         <v>201</v>
       </c>
-      <c r="F49" s="27" t="s">
+      <c r="G49" s="20" t="s">
         <v>202</v>
-      </c>
-      <c r="G49" s="20" t="s">
-        <v>203</v>
       </c>
       <c r="H49" s="21"/>
       <c r="I49" s="11"/>
@@ -3584,32 +3587,32 @@
       <c r="L49" s="11"/>
       <c r="M49" s="11"/>
       <c r="N49" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O49" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P49" s="11"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="6">
         <v>24</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C50" s="15"/>
       <c r="D50" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="E50" s="36" t="s">
         <v>204</v>
       </c>
-      <c r="E50" s="37" t="s">
+      <c r="F50" s="27" t="s">
         <v>205</v>
       </c>
-      <c r="F50" s="27" t="s">
-        <v>206</v>
-      </c>
       <c r="G50" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H50" s="21"/>
       <c r="I50" s="11"/>
@@ -3620,32 +3623,32 @@
       <c r="L50" s="11"/>
       <c r="M50" s="11"/>
       <c r="N50" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O50" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P50" s="11"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="6">
         <v>25</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C51" s="15"/>
       <c r="D51" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="E51" s="36" t="s">
         <v>207</v>
       </c>
-      <c r="E51" s="37" t="s">
+      <c r="F51" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="F51" s="27" t="s">
-        <v>209</v>
-      </c>
       <c r="G51" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H51" s="21"/>
       <c r="I51" s="11"/>
@@ -3656,32 +3659,32 @@
       <c r="L51" s="11"/>
       <c r="M51" s="11"/>
       <c r="N51" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O51" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P51" s="11"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="6">
         <v>26</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C52" s="7"/>
       <c r="D52" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E52" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="E52" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="F52" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="F52" s="27" t="s">
-        <v>212</v>
-      </c>
       <c r="G52" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H52" s="21"/>
       <c r="I52" s="11"/>
@@ -3692,34 +3695,34 @@
       <c r="L52" s="11"/>
       <c r="M52" s="11"/>
       <c r="N52" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O52" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P52" s="11"/>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E53" s="36" t="s">
         <v>213</v>
       </c>
-      <c r="B53" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D53" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E53" s="37" t="s">
+      <c r="F53" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="F53" s="27" t="s">
-        <v>215</v>
-      </c>
       <c r="G53" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H53" s="21"/>
       <c r="I53" s="11"/>
@@ -3730,34 +3733,34 @@
       <c r="L53" s="11"/>
       <c r="M53" s="11"/>
       <c r="N53" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O53" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P53" s="11"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E54" s="36" t="s">
         <v>216</v>
       </c>
-      <c r="B54" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D54" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E54" s="37" t="s">
+      <c r="F54" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="F54" s="27" t="s">
-        <v>218</v>
-      </c>
       <c r="G54" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H54" s="21"/>
       <c r="I54" s="11"/>
@@ -3768,34 +3771,34 @@
       <c r="L54" s="11"/>
       <c r="M54" s="11"/>
       <c r="N54" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O54" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P54" s="11"/>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D55" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E55" s="36" t="s">
         <v>219</v>
       </c>
-      <c r="B55" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D55" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E55" s="37" t="s">
+      <c r="F55" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="F55" s="27" t="s">
-        <v>221</v>
-      </c>
       <c r="G55" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H55" s="21"/>
       <c r="I55" s="11"/>
@@ -3806,34 +3809,34 @@
       <c r="L55" s="11"/>
       <c r="M55" s="11"/>
       <c r="N55" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O55" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P55" s="11"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E56" s="36" t="s">
         <v>222</v>
       </c>
-      <c r="B56" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D56" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E56" s="37" t="s">
+      <c r="F56" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="F56" s="27" t="s">
-        <v>224</v>
-      </c>
       <c r="G56" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H56" s="21"/>
       <c r="I56" s="11"/>
@@ -3844,34 +3847,34 @@
       <c r="L56" s="11"/>
       <c r="M56" s="11"/>
       <c r="N56" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O56" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P56" s="11"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E57" s="36" t="s">
         <v>225</v>
       </c>
-      <c r="B57" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D57" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E57" s="37" t="s">
+      <c r="F57" s="27" t="s">
         <v>226</v>
       </c>
-      <c r="F57" s="27" t="s">
-        <v>227</v>
-      </c>
       <c r="G57" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H57" s="21"/>
       <c r="I57" s="11"/>
@@ -3882,34 +3885,34 @@
       <c r="L57" s="11"/>
       <c r="M57" s="11"/>
       <c r="N57" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O57" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P57" s="11"/>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E58" s="36" t="s">
         <v>228</v>
       </c>
-      <c r="B58" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D58" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E58" s="37" t="s">
+      <c r="F58" s="27" t="s">
         <v>229</v>
       </c>
-      <c r="F58" s="27" t="s">
-        <v>230</v>
-      </c>
       <c r="G58" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H58" s="21"/>
       <c r="I58" s="11"/>
@@ -3920,32 +3923,32 @@
       <c r="L58" s="11"/>
       <c r="M58" s="11"/>
       <c r="N58" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O58" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P58" s="11"/>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C59" s="7"/>
       <c r="D59" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="E59" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E59" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="F59" s="27" t="s">
         <v>232</v>
       </c>
-      <c r="F59" s="27" t="s">
-        <v>233</v>
-      </c>
       <c r="G59" s="20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H59" s="21"/>
       <c r="I59" s="11"/>
@@ -3956,34 +3959,34 @@
       <c r="L59" s="11"/>
       <c r="M59" s="11"/>
       <c r="N59" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O59" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P59" s="11"/>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E60" s="36" t="s">
         <v>234</v>
       </c>
-      <c r="B60" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C60" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D60" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E60" s="37" t="s">
+      <c r="F60" s="27" t="s">
         <v>235</v>
       </c>
-      <c r="F60" s="27" t="s">
-        <v>236</v>
-      </c>
       <c r="G60" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H60" s="21"/>
       <c r="I60" s="11"/>
@@ -3994,34 +3997,34 @@
       <c r="L60" s="11"/>
       <c r="M60" s="11"/>
       <c r="N60" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O60" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P60" s="11"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D61" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E61" s="36" t="s">
         <v>237</v>
       </c>
-      <c r="B61" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D61" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E61" s="37" t="s">
+      <c r="F61" s="27" t="s">
         <v>238</v>
       </c>
-      <c r="F61" s="27" t="s">
-        <v>239</v>
-      </c>
       <c r="G61" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H61" s="21"/>
       <c r="I61" s="11"/>
@@ -4032,32 +4035,32 @@
       <c r="L61" s="11"/>
       <c r="M61" s="11"/>
       <c r="N61" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O61" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P61" s="11"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="6">
         <v>32</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C62" s="7"/>
       <c r="D62" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="E62" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="E62" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="F62" s="29" t="s">
         <v>240</v>
       </c>
-      <c r="F62" s="29" t="s">
-        <v>241</v>
-      </c>
       <c r="G62" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H62" s="21"/>
       <c r="I62" s="11"/>
@@ -4068,32 +4071,32 @@
       <c r="L62" s="11"/>
       <c r="M62" s="11"/>
       <c r="N62" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O62" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P62" s="11"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="17" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C63" s="7"/>
       <c r="D63" s="28" t="s">
-        <v>110</v>
-      </c>
-      <c r="E63" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="E63" s="36" t="s">
+        <v>242</v>
+      </c>
+      <c r="F63" s="29" t="s">
         <v>243</v>
       </c>
-      <c r="F63" s="29" t="s">
-        <v>244</v>
-      </c>
       <c r="G63" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H63" s="21"/>
       <c r="I63" s="11"/>
@@ -4104,32 +4107,32 @@
       <c r="L63" s="11"/>
       <c r="M63" s="11"/>
       <c r="N63" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O63" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P63" s="11"/>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="17" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C64" s="7"/>
       <c r="D64" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="E64" s="37" t="s">
-        <v>246</v>
+        <v>113</v>
+      </c>
+      <c r="E64" s="36" t="s">
+        <v>245</v>
       </c>
       <c r="F64" s="29" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G64" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H64" s="21"/>
       <c r="I64" s="11"/>
@@ -4140,32 +4143,32 @@
       <c r="L64" s="11"/>
       <c r="M64" s="11"/>
       <c r="N64" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O64" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P64" s="11"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="17" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C65" s="7"/>
       <c r="D65" s="28" t="s">
-        <v>118</v>
-      </c>
-      <c r="E65" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="E65" s="36" t="s">
+        <v>247</v>
+      </c>
+      <c r="F65" s="29" t="s">
         <v>248</v>
       </c>
-      <c r="F65" s="29" t="s">
-        <v>249</v>
-      </c>
       <c r="G65" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H65" s="21"/>
       <c r="I65" s="11"/>
@@ -4176,32 +4179,32 @@
       <c r="L65" s="11"/>
       <c r="M65" s="11"/>
       <c r="N65" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O65" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P65" s="11"/>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="17" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C66" s="7"/>
       <c r="D66" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="E66" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="E66" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="F66" s="29" t="s">
         <v>251</v>
       </c>
-      <c r="F66" s="29" t="s">
-        <v>252</v>
-      </c>
       <c r="G66" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H66" s="21"/>
       <c r="I66" s="11"/>
@@ -4212,32 +4215,32 @@
       <c r="L66" s="11"/>
       <c r="M66" s="11"/>
       <c r="N66" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O66" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P66" s="11"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="6">
         <v>33</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C67" s="7"/>
       <c r="D67" s="31" t="s">
-        <v>125</v>
-      </c>
-      <c r="E67" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="E67" s="36" t="s">
+        <v>252</v>
+      </c>
+      <c r="F67" s="29" t="s">
         <v>253</v>
       </c>
-      <c r="F67" s="29" t="s">
-        <v>254</v>
-      </c>
       <c r="G67" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H67" s="21"/>
       <c r="I67" s="11"/>
@@ -4248,32 +4251,32 @@
       <c r="L67" s="11"/>
       <c r="M67" s="11"/>
       <c r="N67" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O67" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P67" s="11"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="17" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C68" s="7"/>
       <c r="D68" s="31" t="s">
-        <v>129</v>
-      </c>
-      <c r="E68" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="E68" s="36" t="s">
+        <v>255</v>
+      </c>
+      <c r="F68" s="29" t="s">
         <v>256</v>
       </c>
-      <c r="F68" s="29" t="s">
-        <v>257</v>
-      </c>
       <c r="G68" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H68" s="21"/>
       <c r="I68" s="11"/>
@@ -4284,32 +4287,32 @@
       <c r="L68" s="11"/>
       <c r="M68" s="11"/>
       <c r="N68" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O68" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P68" s="11"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C69" s="7"/>
       <c r="D69" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="E69" s="37" t="s">
-        <v>259</v>
+        <v>132</v>
+      </c>
+      <c r="E69" s="36" t="s">
+        <v>258</v>
       </c>
       <c r="F69" s="29" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G69" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H69" s="21"/>
       <c r="I69" s="11"/>
@@ -4320,32 +4323,32 @@
       <c r="L69" s="11"/>
       <c r="M69" s="11"/>
       <c r="N69" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O69" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P69" s="11"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C70" s="7"/>
       <c r="D70" s="30" t="s">
-        <v>137</v>
-      </c>
-      <c r="E70" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="E70" s="36" t="s">
+        <v>260</v>
+      </c>
+      <c r="F70" s="29" t="s">
         <v>261</v>
       </c>
-      <c r="F70" s="29" t="s">
-        <v>262</v>
-      </c>
       <c r="G70" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H70" s="21"/>
       <c r="I70" s="11"/>
@@ -4356,32 +4359,32 @@
       <c r="L70" s="11"/>
       <c r="M70" s="11"/>
       <c r="N70" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O70" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P70" s="11"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="6">
         <v>34</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C71" s="7"/>
       <c r="D71" s="30" t="s">
-        <v>140</v>
-      </c>
-      <c r="E71" s="37" t="s">
+        <v>139</v>
+      </c>
+      <c r="E71" s="36" t="s">
+        <v>262</v>
+      </c>
+      <c r="F71" s="29" t="s">
         <v>263</v>
       </c>
-      <c r="F71" s="29" t="s">
-        <v>264</v>
-      </c>
       <c r="G71" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H71" s="21"/>
       <c r="I71" s="11"/>
@@ -4392,32 +4395,32 @@
       <c r="L71" s="11"/>
       <c r="M71" s="11"/>
       <c r="N71" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O71" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P71" s="11"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C72" s="7"/>
       <c r="D72" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="E72" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E72" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="F72" s="29" t="s">
         <v>266</v>
       </c>
-      <c r="F72" s="29" t="s">
-        <v>267</v>
-      </c>
       <c r="G72" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H72" s="21"/>
       <c r="I72" s="11"/>
@@ -4428,32 +4431,32 @@
       <c r="L72" s="11"/>
       <c r="M72" s="11"/>
       <c r="N72" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O72" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P72" s="11"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="17" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C73" s="7"/>
       <c r="D73" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="E73" s="37" t="s">
-        <v>269</v>
+        <v>147</v>
+      </c>
+      <c r="E73" s="36" t="s">
+        <v>268</v>
       </c>
       <c r="F73" s="29" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G73" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H73" s="21"/>
       <c r="I73" s="11"/>
@@ -4464,32 +4467,32 @@
       <c r="L73" s="11"/>
       <c r="M73" s="11"/>
       <c r="N73" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O73" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P73" s="11"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="17" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C74" s="7"/>
       <c r="D74" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="E74" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="E74" s="36" t="s">
+        <v>270</v>
+      </c>
+      <c r="F74" s="29" t="s">
         <v>271</v>
       </c>
-      <c r="F74" s="29" t="s">
-        <v>272</v>
-      </c>
       <c r="G74" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H74" s="21"/>
       <c r="I74" s="11"/>
@@ -4500,32 +4503,32 @@
       <c r="L74" s="11"/>
       <c r="M74" s="11"/>
       <c r="N74" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O74" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P74" s="11"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="6">
         <v>35</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C75" s="7"/>
       <c r="D75" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="E75" s="37" t="s">
+        <v>154</v>
+      </c>
+      <c r="E75" s="36" t="s">
+        <v>272</v>
+      </c>
+      <c r="F75" s="29" t="s">
         <v>273</v>
       </c>
-      <c r="F75" s="29" t="s">
-        <v>274</v>
-      </c>
       <c r="G75" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H75" s="21"/>
       <c r="I75" s="11"/>
@@ -4536,32 +4539,32 @@
       <c r="L75" s="11"/>
       <c r="M75" s="11"/>
       <c r="N75" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O75" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P75" s="11"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C76" s="7"/>
       <c r="D76" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E76" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="E76" s="36" t="s">
+        <v>275</v>
+      </c>
+      <c r="F76" s="29" t="s">
         <v>276</v>
       </c>
-      <c r="F76" s="29" t="s">
-        <v>277</v>
-      </c>
       <c r="G76" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H76" s="21"/>
       <c r="I76" s="11"/>
@@ -4572,32 +4575,32 @@
       <c r="L76" s="11"/>
       <c r="M76" s="11"/>
       <c r="N76" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O76" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P76" s="11"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C77" s="7"/>
       <c r="D77" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="E77" s="37" t="s">
-        <v>279</v>
+        <v>162</v>
+      </c>
+      <c r="E77" s="36" t="s">
+        <v>278</v>
       </c>
       <c r="F77" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G77" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H77" s="21"/>
       <c r="I77" s="11"/>
@@ -4608,32 +4611,32 @@
       <c r="L77" s="11"/>
       <c r="M77" s="11"/>
       <c r="N77" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O77" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P77" s="11"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="17" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C78" s="7"/>
       <c r="D78" s="30" t="s">
-        <v>167</v>
-      </c>
-      <c r="E78" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="E78" s="36" t="s">
+        <v>280</v>
+      </c>
+      <c r="F78" s="29" t="s">
         <v>281</v>
       </c>
-      <c r="F78" s="29" t="s">
-        <v>282</v>
-      </c>
       <c r="G78" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H78" s="21"/>
       <c r="I78" s="11"/>
@@ -4644,32 +4647,32 @@
       <c r="L78" s="11"/>
       <c r="M78" s="11"/>
       <c r="N78" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O78" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P78" s="11"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="6">
         <v>36</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C79" s="7"/>
       <c r="D79" s="30" t="s">
-        <v>170</v>
-      </c>
-      <c r="E79" s="37" t="s">
+        <v>169</v>
+      </c>
+      <c r="E79" s="36" t="s">
+        <v>282</v>
+      </c>
+      <c r="F79" s="29" t="s">
         <v>283</v>
       </c>
-      <c r="F79" s="29" t="s">
-        <v>284</v>
-      </c>
       <c r="G79" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H79" s="21"/>
       <c r="I79" s="11"/>
@@ -4680,32 +4683,32 @@
       <c r="L79" s="11"/>
       <c r="M79" s="11"/>
       <c r="N79" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O79" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P79" s="11"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C80" s="7"/>
       <c r="D80" s="30" t="s">
-        <v>174</v>
-      </c>
-      <c r="E80" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="E80" s="36" t="s">
+        <v>285</v>
+      </c>
+      <c r="F80" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="F80" s="29" t="s">
-        <v>287</v>
-      </c>
       <c r="G80" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H80" s="21"/>
       <c r="I80" s="11"/>
@@ -4716,32 +4719,32 @@
       <c r="L80" s="11"/>
       <c r="M80" s="11"/>
       <c r="N80" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O80" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P80" s="11"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="17" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C81" s="7"/>
       <c r="D81" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="E81" s="37" t="s">
-        <v>289</v>
+        <v>177</v>
+      </c>
+      <c r="E81" s="36" t="s">
+        <v>288</v>
       </c>
       <c r="F81" s="29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G81" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H81" s="21"/>
       <c r="I81" s="11"/>
@@ -4752,32 +4755,32 @@
       <c r="L81" s="11"/>
       <c r="M81" s="11"/>
       <c r="N81" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O81" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P81" s="11"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="17" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C82" s="7"/>
       <c r="D82" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="E82" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="E82" s="36" t="s">
+        <v>290</v>
+      </c>
+      <c r="F82" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="F82" s="29" t="s">
-        <v>292</v>
-      </c>
       <c r="G82" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H82" s="21"/>
       <c r="I82" s="11"/>
@@ -4788,32 +4791,32 @@
       <c r="L82" s="11"/>
       <c r="M82" s="11"/>
       <c r="N82" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O82" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P82" s="11"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="6">
         <v>37</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C83" s="7"/>
       <c r="D83" s="30" t="s">
-        <v>185</v>
-      </c>
-      <c r="E83" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="E83" s="36" t="s">
+        <v>292</v>
+      </c>
+      <c r="F83" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="F83" s="29" t="s">
-        <v>294</v>
-      </c>
       <c r="G83" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H83" s="21"/>
       <c r="I83" s="11"/>
@@ -4824,32 +4827,32 @@
       <c r="L83" s="11"/>
       <c r="M83" s="11"/>
       <c r="N83" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O83" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P83" s="11"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="17" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C84" s="7"/>
       <c r="D84" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="E84" s="37" t="s">
+        <v>188</v>
+      </c>
+      <c r="E84" s="36" t="s">
+        <v>295</v>
+      </c>
+      <c r="F84" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="F84" s="29" t="s">
-        <v>297</v>
-      </c>
       <c r="G84" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H84" s="21"/>
       <c r="I84" s="11"/>
@@ -4860,32 +4863,32 @@
       <c r="L84" s="11"/>
       <c r="M84" s="11"/>
       <c r="N84" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O84" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P84" s="11"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="17" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C85" s="7"/>
       <c r="D85" s="30" t="s">
-        <v>193</v>
-      </c>
-      <c r="E85" s="37" t="s">
-        <v>299</v>
+        <v>192</v>
+      </c>
+      <c r="E85" s="36" t="s">
+        <v>298</v>
       </c>
       <c r="F85" s="29" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G85" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H85" s="21"/>
       <c r="I85" s="11"/>
@@ -4896,32 +4899,32 @@
       <c r="L85" s="11"/>
       <c r="M85" s="11"/>
       <c r="N85" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O85" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P85" s="11"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C86" s="7"/>
       <c r="D86" s="30" t="s">
-        <v>197</v>
-      </c>
-      <c r="E86" s="37" t="s">
+        <v>196</v>
+      </c>
+      <c r="E86" s="36" t="s">
+        <v>300</v>
+      </c>
+      <c r="F86" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="F86" s="29" t="s">
-        <v>302</v>
-      </c>
       <c r="G86" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H86" s="21"/>
       <c r="I86" s="11"/>
@@ -4932,32 +4935,32 @@
       <c r="L86" s="11"/>
       <c r="M86" s="11"/>
       <c r="N86" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O86" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P86" s="11"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="6">
         <v>38</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C87" s="7"/>
       <c r="D87" s="14" t="s">
-        <v>200</v>
-      </c>
-      <c r="E87" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="E87" s="36" t="s">
+        <v>302</v>
+      </c>
+      <c r="F87" s="27" t="s">
         <v>303</v>
       </c>
-      <c r="F87" s="27" t="s">
-        <v>304</v>
-      </c>
       <c r="G87" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H87" s="21"/>
       <c r="I87" s="11"/>
@@ -4968,32 +4971,32 @@
       <c r="L87" s="11"/>
       <c r="M87" s="11"/>
       <c r="N87" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O87" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P87" s="11"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="6">
         <v>39</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C88" s="15"/>
       <c r="D88" s="16" t="s">
-        <v>204</v>
-      </c>
-      <c r="E88" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="E88" s="36" t="s">
+        <v>304</v>
+      </c>
+      <c r="F88" s="27" t="s">
         <v>305</v>
       </c>
-      <c r="F88" s="27" t="s">
-        <v>306</v>
-      </c>
       <c r="G88" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H88" s="21"/>
       <c r="I88" s="11"/>
@@ -5004,32 +5007,32 @@
       <c r="L88" s="11"/>
       <c r="M88" s="11"/>
       <c r="N88" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O88" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P88" s="11"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="6">
         <v>40</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C89" s="15"/>
       <c r="D89" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="E89" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="E89" s="36" t="s">
+        <v>306</v>
+      </c>
+      <c r="F89" s="27" t="s">
         <v>307</v>
       </c>
-      <c r="F89" s="27" t="s">
-        <v>308</v>
-      </c>
       <c r="G89" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H89" s="21"/>
       <c r="I89" s="11"/>
@@ -5040,32 +5043,32 @@
       <c r="L89" s="11"/>
       <c r="M89" s="11"/>
       <c r="N89" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O89" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P89" s="11"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="6">
         <v>41</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C90" s="7"/>
       <c r="D90" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E90" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="E90" s="36" t="s">
+        <v>309</v>
+      </c>
+      <c r="F90" s="27" t="s">
         <v>310</v>
       </c>
-      <c r="F90" s="27" t="s">
-        <v>311</v>
-      </c>
       <c r="G90" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H90" s="21"/>
       <c r="I90" s="11"/>
@@ -5076,34 +5079,34 @@
       <c r="L90" s="11"/>
       <c r="M90" s="11"/>
       <c r="N90" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O90" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P90" s="11"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D91" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E91" s="36" t="s">
         <v>312</v>
       </c>
-      <c r="B91" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C91" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D91" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E91" s="37" t="s">
+      <c r="F91" s="27" t="s">
         <v>313</v>
       </c>
-      <c r="F91" s="27" t="s">
-        <v>314</v>
-      </c>
       <c r="G91" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H91" s="21"/>
       <c r="I91" s="11"/>
@@ -5114,34 +5117,34 @@
       <c r="L91" s="11"/>
       <c r="M91" s="11"/>
       <c r="N91" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O91" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P91" s="11"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="B92" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C92" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D92" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E92" s="36" t="s">
         <v>315</v>
       </c>
-      <c r="B92" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C92" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D92" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E92" s="37" t="s">
+      <c r="F92" s="27" t="s">
         <v>316</v>
       </c>
-      <c r="F92" s="27" t="s">
-        <v>317</v>
-      </c>
       <c r="G92" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H92" s="21"/>
       <c r="I92" s="11"/>
@@ -5152,34 +5155,34 @@
       <c r="L92" s="11"/>
       <c r="M92" s="11"/>
       <c r="N92" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O92" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P92" s="11"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
+        <v>317</v>
+      </c>
+      <c r="B93" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D93" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E93" s="36" t="s">
         <v>318</v>
       </c>
-      <c r="B93" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C93" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D93" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E93" s="37" t="s">
+      <c r="F93" s="27" t="s">
         <v>319</v>
       </c>
-      <c r="F93" s="27" t="s">
-        <v>320</v>
-      </c>
       <c r="G93" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H93" s="21"/>
       <c r="I93" s="11"/>
@@ -5190,34 +5193,34 @@
       <c r="L93" s="11"/>
       <c r="M93" s="11"/>
       <c r="N93" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O93" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P93" s="11"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="17" t="s">
+        <v>320</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D94" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E94" s="36" t="s">
         <v>321</v>
       </c>
-      <c r="B94" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C94" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D94" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E94" s="37" t="s">
+      <c r="F94" s="27" t="s">
         <v>322</v>
       </c>
-      <c r="F94" s="27" t="s">
-        <v>323</v>
-      </c>
       <c r="G94" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H94" s="21"/>
       <c r="I94" s="11"/>
@@ -5228,34 +5231,34 @@
       <c r="L94" s="11"/>
       <c r="M94" s="11"/>
       <c r="N94" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O94" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P94" s="11"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
+        <v>323</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D95" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E95" s="36" t="s">
         <v>324</v>
       </c>
-      <c r="B95" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C95" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D95" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E95" s="37" t="s">
+      <c r="F95" s="27" t="s">
         <v>325</v>
       </c>
-      <c r="F95" s="27" t="s">
-        <v>326</v>
-      </c>
       <c r="G95" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H95" s="21"/>
       <c r="I95" s="11"/>
@@ -5266,34 +5269,34 @@
       <c r="L95" s="11"/>
       <c r="M95" s="11"/>
       <c r="N95" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O95" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P95" s="11"/>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="17" t="s">
+        <v>326</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D96" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E96" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="B96" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C96" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D96" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E96" s="37" t="s">
+      <c r="F96" s="27" t="s">
         <v>328</v>
       </c>
-      <c r="F96" s="27" t="s">
-        <v>329</v>
-      </c>
       <c r="G96" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H96" s="21"/>
       <c r="I96" s="11"/>
@@ -5304,32 +5307,32 @@
       <c r="L96" s="11"/>
       <c r="M96" s="11"/>
       <c r="N96" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O96" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P96" s="11"/>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97" s="17" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B97" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C97" s="7"/>
       <c r="D97" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="E97" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E97" s="36" t="s">
+        <v>330</v>
+      </c>
+      <c r="F97" s="27" t="s">
         <v>331</v>
       </c>
-      <c r="F97" s="27" t="s">
-        <v>332</v>
-      </c>
       <c r="G97" s="20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H97" s="21"/>
       <c r="I97" s="11"/>
@@ -5340,34 +5343,34 @@
       <c r="L97" s="11"/>
       <c r="M97" s="11"/>
       <c r="N97" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O97" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P97" s="11"/>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98" s="17" t="s">
+        <v>332</v>
+      </c>
+      <c r="B98" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C98" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D98" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E98" s="36" t="s">
         <v>333</v>
       </c>
-      <c r="B98" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C98" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D98" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E98" s="37" t="s">
+      <c r="F98" s="27" t="s">
         <v>334</v>
       </c>
-      <c r="F98" s="27" t="s">
-        <v>335</v>
-      </c>
       <c r="G98" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H98" s="21"/>
       <c r="I98" s="11"/>
@@ -5378,34 +5381,34 @@
       <c r="L98" s="11"/>
       <c r="M98" s="11"/>
       <c r="N98" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O98" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P98" s="11"/>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
+        <v>335</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D99" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E99" s="36" t="s">
         <v>336</v>
       </c>
-      <c r="B99" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C99" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D99" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E99" s="37" t="s">
+      <c r="F99" s="27" t="s">
         <v>337</v>
       </c>
-      <c r="F99" s="27" t="s">
-        <v>338</v>
-      </c>
       <c r="G99" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H99" s="21"/>
       <c r="I99" s="11"/>
@@ -5416,32 +5419,32 @@
       <c r="L99" s="11"/>
       <c r="M99" s="11"/>
       <c r="N99" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O99" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P99" s="11"/>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100" s="6">
         <v>47</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C100" s="7"/>
       <c r="D100" s="28" t="s">
-        <v>110</v>
-      </c>
-      <c r="E100" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="E100" s="36" t="s">
+        <v>338</v>
+      </c>
+      <c r="F100" s="29" t="s">
         <v>339</v>
       </c>
-      <c r="F100" s="29" t="s">
-        <v>340</v>
-      </c>
       <c r="G100" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H100" s="21"/>
       <c r="I100" s="18"/>
@@ -5452,32 +5455,32 @@
       <c r="L100" s="18"/>
       <c r="M100" s="18"/>
       <c r="N100" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O100" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P100" s="18"/>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101" s="6">
         <v>48</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C101" s="7"/>
       <c r="D101" s="31" t="s">
-        <v>129</v>
-      </c>
-      <c r="E101" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="E101" s="36" t="s">
+        <v>340</v>
+      </c>
+      <c r="F101" s="29" t="s">
         <v>341</v>
       </c>
-      <c r="F101" s="29" t="s">
-        <v>342</v>
-      </c>
       <c r="G101" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H101" s="21"/>
       <c r="I101" s="18"/>
@@ -5488,32 +5491,32 @@
       <c r="L101" s="18"/>
       <c r="M101" s="18"/>
       <c r="N101" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O101" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P101" s="18"/>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102" s="6">
         <v>49</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C102" s="7"/>
       <c r="D102" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="E102" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E102" s="36" t="s">
+        <v>342</v>
+      </c>
+      <c r="F102" s="29" t="s">
         <v>343</v>
       </c>
-      <c r="F102" s="29" t="s">
-        <v>344</v>
-      </c>
       <c r="G102" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H102" s="21"/>
       <c r="I102" s="18"/>
@@ -5524,32 +5527,32 @@
       <c r="L102" s="18"/>
       <c r="M102" s="18"/>
       <c r="N102" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O102" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P102" s="18"/>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103" s="6">
         <v>50</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C103" s="7"/>
       <c r="D103" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="E103" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="E103" s="36" t="s">
+        <v>344</v>
+      </c>
+      <c r="F103" s="29" t="s">
         <v>345</v>
       </c>
-      <c r="F103" s="29" t="s">
-        <v>346</v>
-      </c>
       <c r="G103" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H103" s="21"/>
       <c r="I103" s="18"/>
@@ -5560,32 +5563,32 @@
       <c r="L103" s="18"/>
       <c r="M103" s="18"/>
       <c r="N103" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O103" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P103" s="18"/>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104" s="6">
         <v>51</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C104" s="7"/>
       <c r="D104" s="30" t="s">
-        <v>174</v>
-      </c>
-      <c r="E104" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="E104" s="36" t="s">
+        <v>346</v>
+      </c>
+      <c r="F104" s="29" t="s">
         <v>347</v>
       </c>
-      <c r="F104" s="29" t="s">
-        <v>348</v>
-      </c>
       <c r="G104" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H104" s="21"/>
       <c r="I104" s="18"/>
@@ -5596,32 +5599,32 @@
       <c r="L104" s="18"/>
       <c r="M104" s="18"/>
       <c r="N104" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O104" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P104" s="18"/>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105" s="6">
         <v>52</v>
       </c>
       <c r="B105" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C105" s="7"/>
       <c r="D105" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="E105" s="37" t="s">
+        <v>188</v>
+      </c>
+      <c r="E105" s="36" t="s">
+        <v>348</v>
+      </c>
+      <c r="F105" s="29" t="s">
         <v>349</v>
       </c>
-      <c r="F105" s="29" t="s">
-        <v>350</v>
-      </c>
       <c r="G105" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H105" s="21"/>
       <c r="I105" s="18"/>
@@ -5632,32 +5635,32 @@
       <c r="L105" s="18"/>
       <c r="M105" s="18"/>
       <c r="N105" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O105" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P105" s="18"/>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" s="6">
         <v>53</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C106" s="7"/>
       <c r="D106" s="14" t="s">
-        <v>200</v>
-      </c>
-      <c r="E106" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="E106" s="36" t="s">
+        <v>350</v>
+      </c>
+      <c r="F106" s="27" t="s">
         <v>351</v>
       </c>
-      <c r="F106" s="27" t="s">
-        <v>352</v>
-      </c>
       <c r="G106" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H106" s="21"/>
       <c r="I106" s="18"/>
@@ -5668,32 +5671,32 @@
       <c r="L106" s="18"/>
       <c r="M106" s="18"/>
       <c r="N106" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O106" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P106" s="18"/>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" s="6">
         <v>54</v>
       </c>
       <c r="B107" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C107" s="15"/>
       <c r="D107" s="16" t="s">
-        <v>204</v>
-      </c>
-      <c r="E107" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="E107" s="36" t="s">
+        <v>352</v>
+      </c>
+      <c r="F107" s="27" t="s">
         <v>353</v>
       </c>
-      <c r="F107" s="27" t="s">
-        <v>354</v>
-      </c>
       <c r="G107" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H107" s="21"/>
       <c r="I107" s="18"/>
@@ -5704,32 +5707,32 @@
       <c r="L107" s="18"/>
       <c r="M107" s="18"/>
       <c r="N107" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O107" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P107" s="18"/>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108" s="6">
         <v>55</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C108" s="15"/>
       <c r="D108" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="E108" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="E108" s="36" t="s">
+        <v>354</v>
+      </c>
+      <c r="F108" s="27" t="s">
         <v>355</v>
       </c>
-      <c r="F108" s="27" t="s">
-        <v>356</v>
-      </c>
       <c r="G108" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H108" s="21"/>
       <c r="I108" s="18"/>
@@ -5740,10 +5743,10 @@
       <c r="L108" s="18"/>
       <c r="M108" s="18"/>
       <c r="N108" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O108" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P108" s="18"/>
     </row>

</xml_diff>